<commit_message>
Add columns, hero blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (21):
- AGENTS.md
- PROJECT.md
- blocks/columns/columns.css
- blocks/columns/columns.js
- blocks/hero/hero.css
- blocks/hero/hero.js
- drafts/wknd/index.plain.html
- styles/styles.css
- tools/importer/import-editorial-section-page.bundle.js
- tools/importer/import-editorial-section-page.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/import-hub-landing-page.bundle.js
- tools/importer/import-hub-landing-page.js
- tools/importer/import-informational-page.bundle.js
- tools/importer/import-informational-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/columns-editorial.js -> tools/importer/parsers/columns-numbered.js
- tools/importer/parsers/hero-full.js
- tools/importer/reports/import-editorial-section-page.report.xlsx
- tools/importer/reports/wknd/sustainability.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-editorial-section-page.report.xlsx
+++ b/tools/importer/reports/import-editorial-section-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="114">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -43,6 +49,9 @@
     <t>["hero-full","columns-about","cards-feature","tabs-team","cards-article"]</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>wknd/about</t>
   </si>
   <si>
@@ -103,34 +112,54 @@
     <t>https://gabrielwalt.github.io/wknd/community.html</t>
   </si>
   <si>
+    <t>wknd/destinations.html.report.json</t>
+  </si>
+  <si>
+    <t>CustomImportScript.default not found after 10s. The bundled script may not have loaded correctly. Check browser console for errors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error: CustomImportScript.default not found after 10s. The bundled script may not have loaded correctly. Check browser console for errors.
+    at processUrl (file:///home/node/.excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:293:13)
+    at async main (file:///home/node/.excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:457:22)</t>
+  </si>
+  <si>
+    <t>wknd/destinations.html</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-03-25T23:39:23.930Z</t>
+  </si>
+  <si>
+    <t>https://gabrielwalt.github.io/wknd/destinations.html</t>
+  </si>
+  <si>
     <t>wknd/destinations.report.json</t>
   </si>
   <si>
-    <t>["columns-featured","columns-editorial","cards-article","cards-article","cards-article","cards-article","cards-article","columns-promo"]</t>
+    <t>["hero-full","columns-featured","columns-editorial","cards-article","cards-article","cards-article","cards-article","cards-article","columns-promo"]</t>
   </si>
   <si>
     <t>wknd/destinations</t>
   </si>
   <si>
-    <t>2026-03-25T22:41:34.396Z</t>
+    <t>2026-03-25T23:40:03.762Z</t>
   </si>
   <si>
     <t>Destinations — WKND Adventures</t>
   </si>
   <si>
-    <t>https://gabrielwalt.github.io/wknd/destinations.html</t>
-  </si>
-  <si>
     <t>wknd/expeditions.report.json</t>
   </si>
   <si>
-    <t>["tabs-activity","columns-editorial","columns-editorial","cards-article","columns-promo"]</t>
+    <t>["hero-full","tabs-activity","columns-editorial","columns-editorial","cards-article","columns-promo"]</t>
   </si>
   <si>
     <t>wknd/expeditions</t>
   </si>
   <si>
-    <t>2026-03-25T22:41:30.735Z</t>
+    <t>2026-03-25T23:43:49.103Z</t>
   </si>
   <si>
     <t>Expeditions — WKND Adventures</t>
@@ -178,13 +207,13 @@
     <t>wknd/gear.report.json</t>
   </si>
   <si>
-    <t>["columns-featured","tabs-activity","columns-editorial","cards-article","cards-article","cards-article","cards-article","cards-article"]</t>
+    <t>["hero-full","columns-featured","tabs-activity","columns-editorial","cards-article","cards-article","cards-article","cards-article","cards-article"]</t>
   </si>
   <si>
     <t>wknd/gear</t>
   </si>
   <si>
-    <t>2026-03-25T22:41:38.410Z</t>
+    <t>2026-03-25T23:43:54.566Z</t>
   </si>
   <si>
     <t>Gear — WKND Adventures</t>
@@ -217,13 +246,13 @@
     <t>wknd/sustainability.report.json</t>
   </si>
   <si>
-    <t>["hero-full","columns-featured"]</t>
+    <t>["hero","columns-featured","columns-numbered"]</t>
   </si>
   <si>
     <t>wknd/sustainability</t>
   </si>
   <si>
-    <t>2026-03-25T22:41:49.063Z</t>
+    <t>2026-03-26T00:18:54.671Z</t>
   </si>
   <si>
     <t>Wild Ethics — WKND Adventures</t>
@@ -714,18 +743,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="50" customWidth="1"/>
+    <col min="2" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -750,425 +779,559 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" t="s">
-        <v>56</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" t="s">
-        <v>62</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>63</v>
-      </c>
-      <c r="F10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" t="s">
-        <v>65</v>
       </c>
       <c r="H10" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="I11" t="s">
+        <v>74</v>
+      </c>
+      <c r="J11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F12" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="H12" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G13" t="s">
+        <v>85</v>
+      </c>
+      <c r="H13" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" t="s">
+        <v>87</v>
+      </c>
+      <c r="J13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" t="s">
         <v>83</v>
       </c>
-      <c r="H13" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
         <v>85</v>
       </c>
-      <c r="B14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>76</v>
-      </c>
-      <c r="F14" t="s">
-        <v>87</v>
-      </c>
-      <c r="G14" t="s">
-        <v>88</v>
-      </c>
       <c r="H14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="I14" t="s">
+        <v>92</v>
+      </c>
+      <c r="J14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="F15" t="s">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="H15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="I15" t="s">
+        <v>97</v>
+      </c>
+      <c r="J15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>97</v>
+        <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="H16" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+      <c r="I16" t="s">
+        <v>102</v>
+      </c>
+      <c r="J16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="F17" t="s">
-        <v>102</v>
+        <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="H17" t="s">
-        <v>104</v>
+        <v>106</v>
+      </c>
+      <c r="I17" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" t="s">
+        <v>111</v>
+      </c>
+      <c r="I18" t="s">
+        <v>112</v>
+      </c>
+      <c r="J18" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>